<commit_message>
Update supervision tracker - Ryan Phase 1 and 2 summary added - March 2026
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Supervision sessions/EMDR_Supervision_Tracking_v2.xlsx
+++ b/Supervision sessions/EMDR_Supervision_Tracking_v2.xlsx
@@ -18,9 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd-mmm-yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -56,7 +55,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -78,16 +77,60 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -101,6 +144,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -525,7 +573,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="8" t="n">
         <v>45993</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -561,7 +609,7 @@
       <c r="I2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="8" t="n">
         <v>46028</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -593,7 +641,7 @@
       <c r="I3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="8" t="n">
         <v>46041</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -630,7 +678,7 @@
       <c r="I4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="8" t="n">
         <v>46056</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -666,7 +714,7 @@
       <c r="I5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="8" t="n">
         <v>46072</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -698,7 +746,7 @@
       <c r="I6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="8" t="n">
         <v>46084</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -717,7 +765,8 @@
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Christina
-Sharon</t>
+Sharon
+Ryan</t>
         </is>
       </c>
       <c r="F7" s="3">
@@ -735,7 +784,7 @@
       <c r="I7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="8" t="n">
         <v>46100</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -767,7 +816,7 @@
       <c r="I8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="8" t="n">
         <v>46126</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -803,7 +852,7 @@
       <c r="I9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="8" t="n">
         <v>46131</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -835,7 +884,7 @@
       <c r="I10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="8" t="n">
         <v>46147</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -867,7 +916,7 @@
       <c r="I11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="8" t="n">
         <v>46161</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -899,7 +948,7 @@
       <c r="I12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="8" t="n">
         <v>46175</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -931,7 +980,7 @@
       <c r="I13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="8" t="n">
         <v>46192</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -963,7 +1012,7 @@
       <c r="I14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="8" t="n">
         <v>46210</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -995,7 +1044,7 @@
       <c r="I15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="8" t="n">
         <v>46222</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1027,7 +1076,7 @@
       <c r="I16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="8" t="n">
         <v>46253</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1059,7 +1108,7 @@
       <c r="I17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="8" t="n">
         <v>46266</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1091,7 +1140,7 @@
       <c r="I18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="8" t="n">
         <v>46284</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1123,7 +1172,7 @@
       <c r="I19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="8" t="n">
         <v>46301</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1155,7 +1204,7 @@
       <c r="I20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="8" t="n">
         <v>46314</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1187,7 +1236,7 @@
       <c r="I21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="8" t="n">
         <v>46329</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1219,7 +1268,7 @@
       <c r="I22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="8" t="n">
         <v>46345</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1251,7 +1300,7 @@
       <c r="I23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="8" t="n">
         <v>46357</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1283,7 +1332,7 @@
       <c r="I24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="8" t="n">
         <v>46375</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1518,14 +1567,30 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Client 4</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr"/>
+          <t>Ryan</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
       <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1 and 2 - EMDR Supervision Summary (Ryan-spvsn-w-Hannah-3326)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Dr Hannah Bryan</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>03-Mar-2026</t>
+        </is>
+      </c>
       <c r="G5" s="3">
         <f>IF(TRIM(F5)="","",LEN(TRIM(F5))-LEN(SUBSTITUTE(TRIM(F5),CHAR(10),""))+1)</f>
         <v/>
@@ -1534,7 +1599,11 @@
         <f>IF(TRIM(F5)="","",TRIM(RIGHT(SUBSTITUTE(TRIM(F5),CHAR(10),REPT(" ",200)),200)))</f>
         <v/>
       </c>
-      <c r="I5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Focus on present-day cringe memory first per Hannah's supervision guidance.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2007,13 +2076,13 @@
           <t>EMDR Accreditation Tracking Dashboard</t>
         </is>
       </c>
-      <c r="B1" s="5" t="n"/>
-      <c r="C1" s="5" t="n"/>
-      <c r="D1" s="5" t="n"/>
-      <c r="E1" s="5" t="n"/>
-      <c r="F1" s="5" t="n"/>
-      <c r="G1" s="5" t="n"/>
-      <c r="H1" s="5" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="9" t="n"/>
+      <c r="D1" s="9" t="n"/>
+      <c r="E1" s="9" t="n"/>
+      <c r="F1" s="9" t="n"/>
+      <c r="G1" s="9" t="n"/>
+      <c r="H1" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -2209,6 +2278,13 @@
           <t>1) Enter clients presented per session in Supervision Log column E using one client per line (ALT+ENTER).</t>
         </is>
       </c>
+      <c r="B25" s="9" t="n"/>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2216,6 +2292,13 @@
           <t>2) Keep Client Log dates presented (one per line). Times Presented and totals update automatically.</t>
         </is>
       </c>
+      <c r="B26" s="9" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2223,6 +2306,13 @@
           <t>3) Adjust B7 if you want a more realistic client-completion projection.</t>
         </is>
       </c>
+      <c r="B27" s="9" t="n"/>
+      <c r="C27" s="9" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="F27" s="9" t="n"/>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>